<commit_message>
research: checkpoint track-a docs + empirical waves + availability merge
</commit_message>
<xml_diff>
--- a/research/runs/20260228-180047-excel-compat-empirical-pass-01/fixtures/recalc_event_matrix.xlsx
+++ b/research/runs/20260228-180047-excel-compat-empirical-pass-01/fixtures/recalc_event_matrix.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Work\DnaCalc\Foundation\research\runs\20260228-180047-excel-compat-empirical-pass-01\fixtures\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D7FCEF49-EE95-4F99-9DC4-7CB7701839CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA593515-0FAC-4D1A-AB33-0FC8C3AF113B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="7440" yWindow="3075" windowWidth="17460" windowHeight="11595" xr2:uid="{7374BFEE-B1B0-4CD3-BDDC-CEAFF6EF225E}"/>
   </bookViews>
@@ -66,8 +66,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="22" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -406,12 +407,12 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1">
-        <f>SUM(B1:B3)</f>
-        <v>60</v>
+      <c r="A1" s="1">
+        <f>INDEX(B1:B3,2)</f>
+        <v>7</v>
       </c>
       <c r="B1">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="C1">
         <v>111</v>
@@ -419,12 +420,12 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B2">
-        <v>20</v>
+        <v>7</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B3">
-        <v>30</v>
+        <v>9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>